<commit_message>
Day 02: Added Average Sales  and Transactions
Added Average Sales and Count Total Sales Transactions Measure
</commit_message>
<xml_diff>
--- a/Problems.xlsx
+++ b/Problems.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Data Analytics\ReClasses\Power_BI\Practice\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A467F241-0AB7-442E-9D44-C6AE6400D8F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3EA466E5-1271-41EE-97BE-6B27642F9BC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{6D85762D-61CB-4066-BFD6-5FB565DD6CD3}"/>
   </bookViews>
@@ -34,9 +34,15 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1" uniqueCount="1">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
   <si>
     <t>Q.1: Calculate Total Sales Amount</t>
+  </si>
+  <si>
+    <t>Q.2: Calculate Average Unit Price</t>
+  </si>
+  <si>
+    <t>Q.3: Count Total Sales Transactions</t>
   </si>
 </sst>
 </file>
@@ -388,7 +394,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3B0599B9-E571-4B20-A5D2-127E923BB6B4}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:A3"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.35">
@@ -396,6 +402,16 @@
         <v>0</v>
       </c>
     </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>2</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Day-03: Added Q.3 to 9.
 Count Total Sales Transactions
 Find the Highest and Lowest Unit Price
 Calculate Total Quantity Sold
 Count Unique Customers
 Count Missing Discount Values Using COUNTBLANK()
 Calculate Average Sales Amount Per Transaction Using AVERAGEX()
 Find the Highest and Lowest Sales Amount Using MAXX() and MINX()
</commit_message>
<xml_diff>
--- a/Problems.xlsx
+++ b/Problems.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Data Analytics\ReClasses\Power_BI\Practice\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3EA466E5-1271-41EE-97BE-6B27642F9BC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5534DF3B-0DB0-419D-8B78-BCF7C1993E76}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{6D85762D-61CB-4066-BFD6-5FB565DD6CD3}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
   <si>
     <t>Q.1: Calculate Total Sales Amount</t>
   </si>
@@ -43,6 +43,24 @@
   </si>
   <si>
     <t>Q.3: Count Total Sales Transactions</t>
+  </si>
+  <si>
+    <t>Q.4: Find the Highest and Lowest Unit Price</t>
+  </si>
+  <si>
+    <t>Q.5: Calculate Total Quantity Sold</t>
+  </si>
+  <si>
+    <t>Q.6: Count Unique Customers</t>
+  </si>
+  <si>
+    <t>Q.7: Count Missing Discount Values Using COUNTBLANK()</t>
+  </si>
+  <si>
+    <t>Q.8: Calculate Average Sales Amount Per Transaction Using AVERAGEX()</t>
+  </si>
+  <si>
+    <t>Q.9: Find the Highest and Lowest Sales Amount Using MAXX() and MINX()</t>
   </si>
 </sst>
 </file>
@@ -394,7 +412,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3B0599B9-E571-4B20-A5D2-127E923BB6B4}">
-  <dimension ref="A1:A3"/>
+  <dimension ref="A1:A9"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.35">
@@ -412,6 +430,36 @@
         <v>2</v>
       </c>
     </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>8</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Day-04: Added Q.10 to 13.
Calculate the Product of Discount Multipliers Using PRODUCT()  and PRODUCTX()
Count Non-Blank Product IDs Using COUNTA()
Count Transactions with Quantity Greater Than 3 Using COUNTX()
Calculate Total Discount Amount Using SUMX()
</commit_message>
<xml_diff>
--- a/Problems.xlsx
+++ b/Problems.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Data Analytics\ReClasses\Power_BI\Practice\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5534DF3B-0DB0-419D-8B78-BCF7C1993E76}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6DE0649B-BD45-4F89-B36A-93393FA2E623}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{6D85762D-61CB-4066-BFD6-5FB565DD6CD3}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
   <si>
     <t>Q.1: Calculate Total Sales Amount</t>
   </si>
@@ -61,6 +61,18 @@
   </si>
   <si>
     <t>Q.9: Find the Highest and Lowest Sales Amount Using MAXX() and MINX()</t>
+  </si>
+  <si>
+    <t>Q.10: Calculate the Product of Discount Multipliers Using PRODUCT()  and PRODUCTX()</t>
+  </si>
+  <si>
+    <t>Q.11: Count Non-Blank Product IDs Using COUNTA()</t>
+  </si>
+  <si>
+    <t>Q.12: Count Transactions with Quantity Greater Than 3 Using COUNTX()</t>
+  </si>
+  <si>
+    <t>Q.13: Calculate Total Discount Amount Using SUMX()</t>
   </si>
 </sst>
 </file>
@@ -412,7 +424,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3B0599B9-E571-4B20-A5D2-127E923BB6B4}">
-  <dimension ref="A1:A9"/>
+  <dimension ref="A1:A13"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.35">
@@ -460,6 +472,26 @@
         <v>8</v>
       </c>
     </row>
+    <row r="10" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
+        <v>12</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Day-05: Added 4 Questions.
 Count Products Sold More then once Using DISTINCT COUNT()
 Calculate Net Sales Amount After Discount
 Calculate Total Sales for the North Region Using CALCULATE()
 Calculate High-Value Sales Using FILTERS()
</commit_message>
<xml_diff>
--- a/Problems.xlsx
+++ b/Problems.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Data Analytics\ReClasses\Power_BI\Practice\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6DE0649B-BD45-4F89-B36A-93393FA2E623}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93B647EF-4444-4755-9FFC-C9DED00619DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{6D85762D-61CB-4066-BFD6-5FB565DD6CD3}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{6D85762D-61CB-4066-BFD6-5FB565DD6CD3}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Beginner" sheetId="1" r:id="rId1"/>
+    <sheet name="Intermediate" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -34,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
   <si>
     <t>Q.1: Calculate Total Sales Amount</t>
   </si>
@@ -73,6 +74,24 @@
   </si>
   <si>
     <t>Q.13: Calculate Total Discount Amount Using SUMX()</t>
+  </si>
+  <si>
+    <t>Q.14: Count Products Sold More then once Using DISTINCT COUNT()</t>
+  </si>
+  <si>
+    <t>Q.15: Calculate Net Sales Amount After Discount</t>
+  </si>
+  <si>
+    <t>Beginner Practice Questions</t>
+  </si>
+  <si>
+    <t>Intermediate Practice Questions</t>
+  </si>
+  <si>
+    <t>Q.1: Calculate Total Sales for the North Region Using CALCULATE()</t>
+  </si>
+  <si>
+    <t>Q.2: Calculate High-Value Sales Using FILTERS()</t>
   </si>
 </sst>
 </file>
@@ -424,72 +443,112 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3B0599B9-E571-4B20-A5D2-127E923BB6B4}">
-  <dimension ref="A1:A13"/>
+  <dimension ref="A1:A16"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>0</v>
+        <v>15</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="14" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
         <v>12</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
+        <v>14</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E16DE348-3DD1-4281-9113-63A82C592DA5}">
+  <dimension ref="A1:A3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>18</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Day-06: Added 4 Questions.
 Calculate Percentage Of Total Sales Using ALL()
 Calculate Regional Sales While Perserving Product Category Filter Using ALLEXCEPT()
 Calculate Visual Total Sales Using ALLSELECTED()
 Calculate Electronics Sales Using CALCULATE() and FILTER()
</commit_message>
<xml_diff>
--- a/Problems.xlsx
+++ b/Problems.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Data Analytics\ReClasses\Power_BI\Practice\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93B647EF-4444-4755-9FFC-C9DED00619DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61048501-42E1-48F4-BE8C-2D9E474B1132}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{6D85762D-61CB-4066-BFD6-5FB565DD6CD3}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
   <si>
     <t>Q.1: Calculate Total Sales Amount</t>
   </si>
@@ -92,6 +92,18 @@
   </si>
   <si>
     <t>Q.2: Calculate High-Value Sales Using FILTERS()</t>
+  </si>
+  <si>
+    <t>Q.3: Calculate Percentage Of Total Sales Using ALL()</t>
+  </si>
+  <si>
+    <t>Q.4: Calculate Regional Sales While Perserving Product Category Filter Using ALLEXCEPT()</t>
+  </si>
+  <si>
+    <t>Q.5: Calculate Visual Total Sales Using ALLSELECTED()</t>
+  </si>
+  <si>
+    <t>Q.6: Calculate Electronics Sales Using CALCULATE() and FILTER()</t>
   </si>
 </sst>
 </file>
@@ -533,7 +545,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E16DE348-3DD1-4281-9113-63A82C592DA5}">
-  <dimension ref="A1:A3"/>
+  <dimension ref="A1:A7"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.35">
@@ -551,6 +563,26 @@
         <v>18</v>
       </c>
     </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>22</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Day-07: Added 3  Questions.
Calculate Top Selling Product Sales Using SELECTEDVALUE()
Calculate Product Rank Using RANK()
Retrieve Sales Rank Within Each Region Using RANK () and PARTITIONBY()
</commit_message>
<xml_diff>
--- a/Problems.xlsx
+++ b/Problems.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Data Analytics\ReClasses\Power_BI\Practice\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61048501-42E1-48F4-BE8C-2D9E474B1132}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F7551E6-58FF-45BF-9F0D-B266A3FEAE6E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{6D85762D-61CB-4066-BFD6-5FB565DD6CD3}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="28">
   <si>
     <t>Q.1: Calculate Total Sales Amount</t>
   </si>
@@ -104,6 +104,21 @@
   </si>
   <si>
     <t>Q.6: Calculate Electronics Sales Using CALCULATE() and FILTER()</t>
+  </si>
+  <si>
+    <t>Q.7: Calculate Top Selling Product Sales Using SELECTEDVALUE()</t>
+  </si>
+  <si>
+    <t>Q.8: Retrieve Product Cost Price Using LOOKUPVALUE()(Not Done)</t>
+  </si>
+  <si>
+    <t>Q.9: Calculate Previous Transaction Sales Using OFFSET()(Not Done)</t>
+  </si>
+  <si>
+    <t>Q.10: Calculate Product Rank Using RANK()</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Q.11: Retrieve Sales Rank Within Each Region Using RANK () and PARTITIONBY() </t>
   </si>
 </sst>
 </file>
@@ -545,7 +560,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E16DE348-3DD1-4281-9113-63A82C592DA5}">
-  <dimension ref="A1:A7"/>
+  <dimension ref="A1:A12"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.35">
@@ -583,6 +598,31 @@
         <v>22</v>
       </c>
     </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>27</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Day-08: Added 3 Questions.
 Retrieve Customer Sales Using RELATED()
 Calculate Total Sales for Each Cutomer Using RELATEDTABLE()
 Calculate Customer Lifetime (CLV) Using CALCULATE()
</commit_message>
<xml_diff>
--- a/Problems.xlsx
+++ b/Problems.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Data Analytics\ReClasses\Power_BI\Practice\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F7551E6-58FF-45BF-9F0D-B266A3FEAE6E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C96BAD5C-8B9A-4E26-9881-C610646AFD80}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{6D85762D-61CB-4066-BFD6-5FB565DD6CD3}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="32">
   <si>
     <t>Q.1: Calculate Total Sales Amount</t>
   </si>
@@ -119,6 +119,18 @@
   </si>
   <si>
     <t xml:space="preserve">Q.11: Retrieve Sales Rank Within Each Region Using RANK () and PARTITIONBY() </t>
+  </si>
+  <si>
+    <t>Q.12: Retrieve the Next Transaction Using INDEX()(Not Done)</t>
+  </si>
+  <si>
+    <t>Q.13: Retrieve Customer Sales Using RELATED()</t>
+  </si>
+  <si>
+    <t>Q.14: Calculate Total Sales for Each Cutomer Using RELATEDTABLE()</t>
+  </si>
+  <si>
+    <t>Q.15: Calculate Customer Lifetime (CLV) Using CALCULATE()</t>
   </si>
 </sst>
 </file>
@@ -560,7 +572,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E16DE348-3DD1-4281-9113-63A82C592DA5}">
-  <dimension ref="A1:A12"/>
+  <dimension ref="A1:A16"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.35">
@@ -623,6 +635,26 @@
         <v>27</v>
       </c>
     </row>
+    <row r="13" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="14" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
+        <v>31</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Day-09: Added 3 Questions.
</commit_message>
<xml_diff>
--- a/Problems.xlsx
+++ b/Problems.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Data Analytics\ReClasses\Power_BI\Practice\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C96BAD5C-8B9A-4E26-9881-C610646AFD80}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{944F4C8C-09F2-4D37-BB78-D7A5BE0C3703}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{6D85762D-61CB-4066-BFD6-5FB565DD6CD3}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="2" xr2:uid="{6D85762D-61CB-4066-BFD6-5FB565DD6CD3}"/>
   </bookViews>
   <sheets>
     <sheet name="Beginner" sheetId="1" r:id="rId1"/>
     <sheet name="Intermediate" sheetId="2" r:id="rId2"/>
+    <sheet name="Advanced" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -35,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="37">
   <si>
     <t>Q.1: Calculate Total Sales Amount</t>
   </si>
@@ -131,6 +132,21 @@
   </si>
   <si>
     <t>Q.15: Calculate Customer Lifetime (CLV) Using CALCULATE()</t>
+  </si>
+  <si>
+    <t>Advanced Practice Questions</t>
+  </si>
+  <si>
+    <t>Q.1: Calculate Year-to-Date (YTD) Sales Using CALCULATE() and DATESTYD()</t>
+  </si>
+  <si>
+    <t>Q.2: Calculate Month-to-Date (MTD) Sales Using CALCULATED() and DATESMTD()</t>
+  </si>
+  <si>
+    <t>Q.3: Calculate Quarter-to-Date (QTD) Sales Using CALCULATE() and DATESQTD()</t>
+  </si>
+  <si>
+    <t>Q.4: Calculate Previous Year Sales Using SAMEPERIOD-LAST YEAR()</t>
   </si>
 </sst>
 </file>
@@ -658,4 +674,39 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{957F8A97-C0C4-4373-B1D4-9DC47333A2C6}">
+  <dimension ref="A1:A5"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>36</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>